<commit_message>
xiao 2L complete: SW2+SW6 restored, routed 100%, production packages regenerated
Final routed board: 880 tracks, 186 vias, 70 footprints -- 0 DRC errors,
0 unconnected (kicad-cli DRC + pcbnew ratsnest agree).

- SW2 on XIAO pad 23 (the GPIO freed by the expander removal), fw INPUT_PULLUP.
- SW6 as hardware motor kill via TB6612 STBY gate (R55 10k pull-up, PCM12
  slide shorts STBY to GND); MOT KILL/RUN silkscreen.
- 19 THT axial resistors at beam-clear top-side spots; H1-H4 3.2mm NPTH
  mounting holes restored; no SMD parts on the bottom side (B.Paste empty,
  validator updated accordingly).
- GND closed with refereed stitching: via-in-pad at U2 pin 18 slot midpoint,
  C8.2 escape corridor, ribbon-to-main weld via under the GND diagonal.
- production_2layer/{jlcpcb,lioncircuits} regenerated: 27 BOM lines (12 THT
  hand-solder), 63 CPL placements, 9-layer gerbers + NPTH drills verified,
  all JLC schema gates PASS.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pcb/JLCPCB_2layers_simplified/xiao_linefollower/production_2layer/jlcpcb/BOM_JLC-assembly.xlsx
+++ b/pcb/JLCPCB_2layers_simplified/xiao_linefollower/production_2layer/jlcpcb/BOM_JLC-assembly.xlsx
@@ -62,7 +62,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C1,C4,C11,C18</t>
+          <t xml:space="preserve">C1,C4,C11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -84,7 +84,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2,C3,C8,C12,C14,C15,C50</t>
+          <t xml:space="preserve">C2,C3,C8,C12,C14</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -106,7 +106,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">C5</t>
+          <t xml:space="preserve">C5,C10</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -123,748 +123,506 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">10uF</t>
+          <t xml:space="preserve">IR333-A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">C10</t>
+          <t xml:space="preserve">D1,D2,D3,D4,D5,D6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">C_0805_2012Metric</t>
+          <t xml:space="preserve">LED_D5.0mm_IRGrey</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">C15850</t>
+          <t xml:space="preserve">C264290</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">22uF/25V</t>
+          <t xml:space="preserve">1N4148W</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">C16,C17</t>
+          <t xml:space="preserve">D29</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">C_1210_3225Metric</t>
+          <t xml:space="preserve">D_SOD-123</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">C52306</t>
+          <t xml:space="preserve">C83528</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">220uF/16V</t>
+          <t xml:space="preserve">Power LED 0603 red</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">C30</t>
+          <t xml:space="preserve">D30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">CP_Elec_6.3x7.7</t>
+          <t xml:space="preserve">LED_0603_1608Metric</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2887273</t>
+          <t xml:space="preserve">C2286</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">IR333-A</t>
+          <t xml:space="preserve">2.6A/16V PPTC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">D1,D2,D3,D4,D5,D6</t>
+          <t xml:space="preserve">F1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED_D5.0mm_IRGrey</t>
+          <t xml:space="preserve">Fuse_1812_4532Metric</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">C264290</t>
+          <t xml:space="preserve">C16490</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1N4148W</t>
+          <t xml:space="preserve">BATT_IN_2S</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">D29</t>
+          <t xml:space="preserve">J1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">D_SOD-123</t>
+          <t xml:space="preserve">JST_XH_B2B-XH-A_1x02_P2.50mm_Vertical</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">C83528</t>
+          <t xml:space="preserve">C158012</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Power LED 0603 red</t>
+          <t xml:space="preserve">MOTOR_A_N20_ENCODER</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">D30,D33</t>
+          <t xml:space="preserve">J5,J6</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED_0603_1608Metric</t>
+          <t xml:space="preserve">JST_ZH_B6B-ZR_1x06_P1.50mm_Vertical</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2286</t>
+          <t xml:space="preserve">C157984</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">WALL_FL_LED wall-detection indicator</t>
+          <t xml:space="preserve">BATT_IN_XT60</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">D50,D51,D52,D53,D54,D55</t>
+          <t xml:space="preserve">J10</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED_0603_1608Metric</t>
+          <t xml:space="preserve">AMASS_XT60-M_1x02_P7.20mm_Vertical</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">C5875754</t>
+          <t xml:space="preserve">C98733</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.6A/16V PPTC</t>
+          <t xml:space="preserve">4.7uH</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">F1</t>
+          <t xml:space="preserve">L1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fuse_1812_4532Metric</t>
+          <t xml:space="preserve">L_Bourns_SRP4020TA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">C16490</t>
+          <t xml:space="preserve">C2041623</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">BATT_IN_2S</t>
+          <t xml:space="preserve">Q_PMOS reverse guard</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">J1</t>
+          <t xml:space="preserve">Q1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">JST_XH_B2B-XH-A_1x02_P2.50mm_Vertical</t>
+          <t xml:space="preserve">SOT-23</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">C158012</t>
+          <t xml:space="preserve">C150492</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">MOTOR_A_N20_ENCODER</t>
+          <t xml:space="preserve">PT334-6B</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">J5,J6</t>
+          <t xml:space="preserve">Q2,Q3,Q4,Q5,Q6,Q7</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">JST_ZH_B6B-ZR_1x06_P1.50mm_Vertical</t>
+          <t xml:space="preserve">LED_D5.0mm_IRBlack</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">C157984</t>
+          <t xml:space="preserve">C369188</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">BATT_IN_XT60</t>
+          <t xml:space="preserve">BSS138</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">J10</t>
+          <t xml:space="preserve">Q16,Q17,Q18</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMASS_XT60-M_1x02_P7.20mm_Vertical</t>
+          <t xml:space="preserve">SOT-23</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">C98733</t>
+          <t xml:space="preserve">C82045</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.7uH</t>
+          <t xml:space="preserve">MMBT2222A</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">L1,L2</t>
+          <t xml:space="preserve">Q34</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">L_Bourns_SRP4020TA</t>
+          <t xml:space="preserve">SOT-23</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2041623</t>
+          <t xml:space="preserve">C94515</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q_PMOS reverse guard</t>
+          <t xml:space="preserve">100k</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q1</t>
+          <t xml:space="preserve">R1,R62,R63,R64,R69</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-23</t>
+          <t xml:space="preserve">R_Axial_DIN0207_L6.3mm_D2.5mm_P7.62mm_Horizontal</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">C150492</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT334-6B</t>
+          <t xml:space="preserve">47k</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2,Q3,Q4,Q5,Q6,Q7</t>
+          <t xml:space="preserve">R13,R15,R17,R19,R21,R23</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED_D5.0mm_IRBlack</t>
+          <t xml:space="preserve">R_Axial_DIN0207_L6.3mm_D2.5mm_P7.62mm_Horizontal</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">C369188</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSS138</t>
+          <t xml:space="preserve">33</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q16,Q17,Q18</t>
+          <t xml:space="preserve">R14,R16,R18,R20,R22,R24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-23</t>
+          <t xml:space="preserve">R_Axial_DIN0207_L6.3mm_D2.5mm_P7.62mm_Horizontal</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">C82045</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMBT2222A</t>
+          <t xml:space="preserve">10k</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q34</t>
+          <t xml:space="preserve">R55</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-23</t>
+          <t xml:space="preserve">R_Axial_DIN0207_L6.3mm_D2.5mm_P7.62mm_Horizontal</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">C94515</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">100k</t>
+          <t xml:space="preserve">220</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">R1,R62,R63,R64,R69,R73</t>
+          <t xml:space="preserve">R81</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">R_Axial_DIN0207_L6.3mm_D2.5mm_P7.62mm_Horizontal</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">C96346</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">10k</t>
+          <t xml:space="preserve">1k</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">R6,R7,R8,R9,R55</t>
+          <t xml:space="preserve">R82</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">R_Axial_DIN0207_L6.3mm_D2.5mm_P7.62mm_Horizontal</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">C108451</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">47k</t>
+          <t xml:space="preserve">SW_Push</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">R13,R15,R17,R19,R21,R23</t>
+          <t xml:space="preserve">SW1,SW2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">SW_Push_1P1T_NO_CK_KMR2</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17713</t>
+          <t xml:space="preserve">C269272</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">33</t>
+          <t xml:space="preserve">PWR ALL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">R14,R16,R18,R20,R22,R24</t>
+          <t xml:space="preserve">SW5,SW6</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">SW_SPDT_PCM12</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17634</t>
+          <t xml:space="preserve">C221841</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">220k</t>
+          <t xml:space="preserve">AP63203WU-7</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">R70</t>
+          <t xml:space="preserve">U1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">TSOT-23-6</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17556</t>
+          <t xml:space="preserve">C780769</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">110k</t>
+          <t xml:space="preserve">TB6612FNG</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">R71</t>
+          <t xml:space="preserve">U2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">SSOP-24_5.3x8.2mm_P0.65mm</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2907221</t>
+          <t xml:space="preserve">C141517</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">11k</t>
+          <t xml:space="preserve">Seeed XIAO nRF52840 Sense Plus</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">R74</t>
+          <t xml:space="preserve">U3</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">XIAO-nRF52840-Plus-SMD</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17429</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">220</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R81,R105,R106,R107,R108,R109,R110</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C17557</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1k</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R82,R84</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C17513</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40.2k</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R85</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
           <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.2k</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R103,R104</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C17512</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW_Push</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW1,SW2</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW_Push_1P1T_NO_CK_KMR2</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C269272</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PWR ALL</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW5,SW6,SW7</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW_SPDT_PCM12</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C221841</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AP63203WU-7</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U1</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TSOT-23-6</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C780769</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TB6612FNG</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U2</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SSOP-24_5.3x8.2mm_P0.65mm</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C141517</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Seeed XIAO nRF52840 Sense Plus</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U3</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">XIAO-nRF52840-Plus-SMD</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PCF8574DWR</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U5</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SOIC-16W_7.5x10.3mm_P1.27mm</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C2652271</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TPS54302DDCR</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U7</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SOT-23-6</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C311983</t>
         </is>
       </c>
     </row>

</xml_diff>